<commit_message>
dockerfile: minizinc inclusion fixed updated doku install.sh fixed: DON'T apt-get docker.io
</commit_message>
<xml_diff>
--- a/backend/src/test/resources/csv_import/karrierekompass-linz-2026/Referenten_und_Vorträge_Jürgenxlsx.xlsx
+++ b/backend/src/test/resources/csv_import/karrierekompass-linz-2026/Referenten_und_Vorträge_Jürgenxlsx.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kathr\Documents\jessen\Berufsorientierung\KarriereKompassLinz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kreyj/Java/berufsorientierung/KonfPlan/backend/src/test/resources/csv_import/karrierekompass-linz-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28AF858-57FA-4BC6-B1A4-E00154FC9ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9A5C2B-CD8E-7E4C-9880-D10841C5B4B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="16395" windowHeight="10276" activeTab="1" xr2:uid="{FDC18993-A1F0-2C44-A20A-6CB30829136B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="22000" windowHeight="17600" activeTab="1" xr2:uid="{FDC18993-A1F0-2C44-A20A-6CB30829136B}"/>
   </bookViews>
   <sheets>
     <sheet name="Referenten" sheetId="2" r:id="rId1"/>
@@ -1158,7 +1158,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1188,11 +1188,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1532,17 +1530,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC9EF96-C226-A645-BCA0-04270AB57CB2}">
   <dimension ref="A1:I54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="2" width="17.3125" customWidth="1"/>
-    <col min="3" max="3" width="18.6875" customWidth="1"/>
-    <col min="4" max="5" width="17.3125" customWidth="1"/>
-    <col min="6" max="7" width="17.3125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="17.3125" customWidth="1"/>
-    <col min="9" max="9" width="22.8125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="81.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="7" width="17.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21">
+    <row r="1" spans="1:9" ht="23">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1571,7 +1570,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18">
+    <row r="2" spans="1:9" ht="19">
       <c r="A2" s="12" t="s">
         <v>202</v>
       </c>
@@ -1592,7 +1591,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="18">
+    <row r="3" spans="1:9" ht="19">
       <c r="A3" s="12" t="s">
         <v>203</v>
       </c>
@@ -1611,7 +1610,7 @@
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
     </row>
-    <row r="4" spans="1:9" ht="18">
+    <row r="4" spans="1:9" ht="19">
       <c r="A4" s="12" t="s">
         <v>204</v>
       </c>
@@ -1629,7 +1628,7 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:9" ht="18">
+    <row r="5" spans="1:9" ht="19">
       <c r="A5" s="12" t="s">
         <v>205</v>
       </c>
@@ -1647,7 +1646,7 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="18">
+    <row r="6" spans="1:9" ht="19">
       <c r="A6" s="12" t="s">
         <v>206</v>
       </c>
@@ -1664,7 +1663,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" ht="18">
+    <row r="7" spans="1:9" ht="19">
       <c r="A7" s="12" t="s">
         <v>207</v>
       </c>
@@ -1683,7 +1682,7 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:9" ht="18">
+    <row r="8" spans="1:9" ht="19">
       <c r="A8" s="12" t="s">
         <v>208</v>
       </c>
@@ -1700,7 +1699,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="18">
+    <row r="9" spans="1:9" ht="19">
       <c r="A9" s="12" t="s">
         <v>209</v>
       </c>
@@ -1717,7 +1716,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" ht="18">
+    <row r="10" spans="1:9" ht="19">
       <c r="A10" s="12" t="s">
         <v>210</v>
       </c>
@@ -1734,7 +1733,7 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="18">
+    <row r="11" spans="1:9" ht="19">
       <c r="A11" s="12" t="s">
         <v>211</v>
       </c>
@@ -1753,7 +1752,7 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" ht="18">
+    <row r="12" spans="1:9" ht="19">
       <c r="A12" s="12" t="s">
         <v>212</v>
       </c>
@@ -1772,7 +1771,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" ht="18">
+    <row r="13" spans="1:9" ht="19">
       <c r="A13" s="12" t="s">
         <v>213</v>
       </c>
@@ -1791,7 +1790,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" ht="18">
+    <row r="14" spans="1:9" ht="19">
       <c r="A14" s="12" t="s">
         <v>214</v>
       </c>
@@ -1810,7 +1809,7 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="1:9" ht="18">
+    <row r="15" spans="1:9" ht="19">
       <c r="A15" s="12" t="s">
         <v>215</v>
       </c>
@@ -1828,7 +1827,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" spans="1:9" ht="18">
+    <row r="16" spans="1:9" ht="19">
       <c r="A16" s="12" t="s">
         <v>216</v>
       </c>
@@ -1846,7 +1845,7 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="18">
+    <row r="17" spans="1:9" ht="19">
       <c r="A17" s="12" t="s">
         <v>175</v>
       </c>
@@ -1863,7 +1862,7 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="18">
+    <row r="18" spans="1:9" ht="19">
       <c r="A18" s="12" t="s">
         <v>217</v>
       </c>
@@ -1874,7 +1873,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="18">
+    <row r="19" spans="1:9" ht="19">
       <c r="A19" s="12" t="s">
         <v>219</v>
       </c>
@@ -1888,7 +1887,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="18">
+    <row r="20" spans="1:9" ht="19">
       <c r="A20" s="12" t="s">
         <v>220</v>
       </c>
@@ -1902,7 +1901,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="18">
+    <row r="21" spans="1:9" ht="19">
       <c r="A21" s="12" t="s">
         <v>221</v>
       </c>
@@ -1916,7 +1915,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="18">
+    <row r="22" spans="1:9" ht="19">
       <c r="A22" s="12" t="s">
         <v>222</v>
       </c>
@@ -1930,7 +1929,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="18">
+    <row r="23" spans="1:9" ht="19">
       <c r="A23" s="12" t="s">
         <v>149</v>
       </c>
@@ -1944,7 +1943,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="18">
+    <row r="24" spans="1:9" ht="19">
       <c r="A24" s="12" t="s">
         <v>176</v>
       </c>
@@ -1958,7 +1957,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="18">
+    <row r="25" spans="1:9" ht="19">
       <c r="A25" s="12" t="s">
         <v>223</v>
       </c>
@@ -1972,7 +1971,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="18">
+    <row r="26" spans="1:9" ht="19">
       <c r="A26" s="13" t="s">
         <v>225</v>
       </c>
@@ -1986,7 +1985,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="18">
+    <row r="27" spans="1:9" ht="19">
       <c r="A27" s="13" t="s">
         <v>226</v>
       </c>
@@ -1997,7 +1996,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="18">
+    <row r="28" spans="1:9" ht="19">
       <c r="A28" s="13" t="s">
         <v>227</v>
       </c>
@@ -2008,7 +2007,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="18">
+    <row r="29" spans="1:9" ht="19">
       <c r="A29" s="13" t="s">
         <v>215</v>
       </c>
@@ -2022,7 +2021,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="18">
+    <row r="30" spans="1:9" ht="19">
       <c r="A30" s="13" t="s">
         <v>178</v>
       </c>
@@ -2036,7 +2035,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="18">
+    <row r="31" spans="1:9" ht="19">
       <c r="A31" s="13" t="s">
         <v>181</v>
       </c>
@@ -2050,7 +2049,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="18">
+    <row r="32" spans="1:9" ht="19">
       <c r="A32" s="13" t="s">
         <v>178</v>
       </c>
@@ -2064,7 +2063,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="18">
+    <row r="33" spans="1:4" ht="19">
       <c r="A33" s="13" t="s">
         <v>182</v>
       </c>
@@ -2078,7 +2077,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="18">
+    <row r="34" spans="1:4" ht="19">
       <c r="A34" s="13" t="s">
         <v>183</v>
       </c>
@@ -2092,7 +2091,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="18">
+    <row r="35" spans="1:4" ht="19">
       <c r="A35" s="14" t="s">
         <v>184</v>
       </c>
@@ -2106,7 +2105,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="18">
+    <row r="36" spans="1:4" ht="19">
       <c r="A36" s="13" t="s">
         <v>185</v>
       </c>
@@ -2120,7 +2119,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="18">
+    <row r="37" spans="1:4" ht="19">
       <c r="A37" s="13" t="s">
         <v>186</v>
       </c>
@@ -2134,7 +2133,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="18">
+    <row r="38" spans="1:4" ht="19">
       <c r="A38" s="13" t="s">
         <v>187</v>
       </c>
@@ -2145,7 +2144,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="18">
+    <row r="39" spans="1:4" ht="19">
       <c r="A39" s="13" t="s">
         <v>188</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="18">
+    <row r="40" spans="1:4" ht="19">
       <c r="A40" s="13" t="s">
         <v>189</v>
       </c>
@@ -2167,7 +2166,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="18">
+    <row r="41" spans="1:4" ht="19">
       <c r="A41" s="13" t="s">
         <v>190</v>
       </c>
@@ -2181,7 +2180,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="18">
+    <row r="42" spans="1:4" ht="19">
       <c r="A42" s="13" t="s">
         <v>191</v>
       </c>
@@ -2192,7 +2191,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18">
+    <row r="43" spans="1:4" ht="19">
       <c r="A43" s="13" t="s">
         <v>192</v>
       </c>
@@ -2206,7 +2205,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="18">
+    <row r="44" spans="1:4" ht="19">
       <c r="A44" s="13" t="s">
         <v>193</v>
       </c>
@@ -2220,7 +2219,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="18">
+    <row r="45" spans="1:4" ht="19">
       <c r="A45" s="13" t="s">
         <v>196</v>
       </c>
@@ -2234,7 +2233,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="18">
+    <row r="46" spans="1:4" ht="19">
       <c r="A46" s="13" t="s">
         <v>195</v>
       </c>
@@ -2248,7 +2247,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="18">
+    <row r="47" spans="1:4" ht="19">
       <c r="A47" s="13" t="s">
         <v>197</v>
       </c>
@@ -2259,7 +2258,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="18">
+    <row r="48" spans="1:4" ht="19">
       <c r="A48" s="13" t="s">
         <v>198</v>
       </c>
@@ -2273,7 +2272,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="18">
+    <row r="49" spans="1:7" ht="19">
       <c r="A49" s="13" t="s">
         <v>199</v>
       </c>
@@ -2284,7 +2283,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="18">
+    <row r="50" spans="1:7" ht="19">
       <c r="A50" s="13" t="s">
         <v>200</v>
       </c>
@@ -2298,7 +2297,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="18">
+    <row r="51" spans="1:7" ht="19">
       <c r="A51" s="13" t="s">
         <v>201</v>
       </c>
@@ -2312,7 +2311,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="18">
+    <row r="52" spans="1:7" ht="19">
       <c r="A52" s="18" t="s">
         <v>304</v>
       </c>
@@ -2329,7 +2328,7 @@
       <c r="F52"/>
       <c r="G52"/>
     </row>
-    <row r="53" spans="1:7" ht="18">
+    <row r="53" spans="1:7" ht="19">
       <c r="A53" s="18" t="s">
         <v>308</v>
       </c>
@@ -2346,7 +2345,7 @@
       <c r="F53"/>
       <c r="G53"/>
     </row>
-    <row r="54" spans="1:7" ht="18">
+    <row r="54" spans="1:7" ht="19">
       <c r="A54" s="18" t="s">
         <v>312</v>
       </c>
@@ -2397,19 +2396,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3609FF0-C2D6-7642-9D7C-00C96E963DC6}">
   <dimension ref="A1:N52"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="32.4375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="32.5" style="3" customWidth="1"/>
     <col min="5" max="8" width="0" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="21" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="23.3125" customWidth="1"/>
-    <col min="11" max="11" width="23.1875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="23.33203125" customWidth="1"/>
+    <col min="11" max="11" width="23.1640625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21">
+    <row r="1" spans="1:14" ht="23">
       <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
@@ -2856,27 +2855,27 @@
         <v>127</v>
       </c>
     </row>
-    <row r="50" spans="3:4" ht="31.5">
+    <row r="50" spans="3:4" ht="34">
       <c r="C50" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="D50" s="24" t="s">
+      <c r="D50" s="22" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="51" spans="3:4" ht="47.25">
+    <row r="51" spans="3:4" ht="51">
       <c r="C51" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="D51" s="24" t="s">
+      <c r="D51" s="22" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="52" spans="3:4">
+    <row r="52" spans="3:4" ht="17">
       <c r="C52" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="D52" s="24" t="s">
+      <c r="D52" s="22" t="s">
         <v>316</v>
       </c>
     </row>
@@ -2906,57 +2905,57 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12BD1686-9621-5343-8CED-A79ACF67F931}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="57.3125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.375" customWidth="1"/>
+    <col min="1" max="1" width="57.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="10" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" ht="17">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" ht="17">
       <c r="A3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="31.5">
+    <row r="4" spans="1:2" ht="34">
       <c r="A4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" ht="17">
       <c r="A5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" ht="17">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>325</v>
       </c>
     </row>
@@ -2964,13 +2963,11 @@
       <c r="A7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="21"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="21"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">

</xml_diff>